<commit_message>
Phase 3 (WIP): continued data, API and setup work
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FkouT5fAgzdcE8NaiFmB4Y
</commit_message>
<xml_diff>
--- a/data/sharepoint/Harbourline-Operations/Procedures/Transformer-Equipment-Specs.xlsx
+++ b/data/sharepoint/Harbourline-Operations/Procedures/Transformer-Equipment-Specs.xlsx
@@ -2045,7 +2045,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>NF-PM10-7A</t>
+          <t>NF-PM10-7NA</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2103,7 +2103,7 @@
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>NF-PM15-7A</t>
+          <t>NF-PM15-7NA</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2161,7 +2161,7 @@
       <c r="A30" s="7" t="n"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>NF-PM25-7A</t>
+          <t>NF-PM25-7NA</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2219,7 +2219,7 @@
       <c r="A31" s="7" t="n"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>LTW-PM25-7L</t>
+          <t>LTW-PM25-7NL</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2277,7 +2277,7 @@
       <c r="A32" s="7" t="n"/>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>NF-PM375-7A</t>
+          <t>NF-PM375-7NA</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2335,7 +2335,7 @@
       <c r="A33" s="7" t="n"/>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>NF-PM50-7A</t>
+          <t>NF-PM50-7NA</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2393,7 +2393,7 @@
       <c r="A34" s="7" t="n"/>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>LTW-PM50-7L</t>
+          <t>LTW-PM50-7NL</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2451,7 +2451,7 @@
       <c r="A35" s="7" t="n"/>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>NF-PM75-7A</t>
+          <t>NF-PM75-7NA</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2509,7 +2509,7 @@
       <c r="A36" s="7" t="n"/>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>NF-PM100-7A</t>
+          <t>NF-PM100-7NA</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2567,7 +2567,7 @@
       <c r="A37" s="7" t="n"/>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>LTW-PM100-7L</t>
+          <t>LTW-PM100-7NL</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2625,7 +2625,7 @@
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>NF-PM167-7A</t>
+          <t>NF-PM167-7NA</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -10822,7 +10822,7 @@
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>NF-PM15-7A</t>
+          <t>NF-PM15-7NA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -10847,25 +10847,25 @@
         <v>0</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P17" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2" t="n">
         <v>12</v>
@@ -10875,7 +10875,7 @@
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>LTW-PM25-7L</t>
+          <t>LTW-PM25-7NL</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -10897,28 +10897,28 @@
         <v>0</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P18" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="2" t="n">
         <v>14</v>
@@ -10928,7 +10928,7 @@
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>NF-PM50-7A</t>
+          <t>NF-PM50-7NA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -10950,28 +10950,28 @@
         <v>0</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P19" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="2" t="n">
         <v>19</v>
@@ -10981,7 +10981,7 @@
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>NF-PM75-7A</t>
+          <t>NF-PM75-7NA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -11003,28 +11003,28 @@
         <v>0</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P20" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="2" t="n">
         <v>13</v>
@@ -11034,7 +11034,7 @@
       <c r="A21" s="7" t="n"/>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>LTW-PM100-7L</t>
+          <t>LTW-PM100-7NL</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -11056,28 +11056,28 @@
         <v>0</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P21" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="2" t="n">
         <v>12</v>

</xml_diff>